<commit_message>
v2: capturas publicadas e OS de exemplo
</commit_message>
<xml_diff>
--- a/docs/OS_exemplo.xlsx
+++ b/docs/OS_exemplo.xlsx
@@ -21,7 +21,7 @@
     <t>ORDEM DE SERVIÇO — MANUTENÇÃO DE CFTV</t>
   </si>
   <si>
-    <t>Gerada em: 30/09/2026 16:22     ·     Período dos dados: 31/08/2026 a 28/09/2026 (última atualização 28/09/2026 20:59)</t>
+    <t>Gerada em: 30/09/2026 16:24     ·     Período dos dados: 31/08/2026 a 28/09/2026 (última atualização 28/09/2026 20:59)</t>
   </si>
   <si>
     <t>Filtros: Garagem: Via Sudeste  ·  Câmera: Todas  ·  Problema: 1+ câmera com problema, 100% Offline</t>
@@ -1452,7 +1452,7 @@
     <t>ORDEM DE SERVIÇO — LEGENDA E INSTRUÇÕES</t>
   </si>
   <si>
-    <t>Gerada em 30/09/2026 16:22. Dados de 31/08/2026 a 28/09/2026; última atualização 28/09/2026 20:59.</t>
+    <t>Gerada em 30/09/2026 16:24. Dados de 31/08/2026 a 28/09/2026; última atualização 28/09/2026 20:59.</t>
   </si>
   <si>
     <t>Status de cada câmera (colunas Câm 21 a Câm 26)</t>
@@ -18936,7 +18936,7 @@
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.45" header="0.2" footer="0.2"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
   <headerFooter>
-    <oddFooter>&amp;L&amp;8Controle de CFTV — Ordem de Serviço&amp;C&amp;8Gerada em 30/09/2026 16:22&amp;R&amp;8Página &amp;P de &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;8Controle de CFTV — Ordem de Serviço&amp;C&amp;8Gerada em 30/09/2026 16:24&amp;R&amp;8Página &amp;P de &amp;N</oddFooter>
   </headerFooter>
 </worksheet>
 </file>

</xml_diff>